<commit_message>
comment-task producer + runner (Descifra 2.10); Morelia tasks 125–144
- select_posts_for_comments.py: selects the posts whose comments are worth buying
  (tagger place + LLM theme + official page + traction), tiered deep/sample task
  file with cost before purchase. Fix: declared comment count lives at
  source.stats.n_comments on the ES doc (top-level is never populated) — reading only
  the top level skipped every post.
- run_comment_tasks.py: one facebook_post_comments run per tier; dry-run default,
  --apply buys and publishes.
- tasks.xlsx: theme morelia_descifra — rows 125/126 (keyword discovery, disabled after
  use), 127–144 recurring page rows; run_searches CURRENT_THEME.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tasks.xlsx
+++ b/tasks.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X135"/>
+  <dimension ref="A1:X155"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="19.6640625" customWidth="1" min="2" max="4"/>
@@ -9266,6 +9266,1064 @@
         <is>
           <t>{"enrich_author_after_likes": 50}</t>
         </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>125</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>facebook_keyword_search</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>morelia_descifra</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Morelia keyword (round 1, discovery)</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>morelia</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="K136" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L136" t="n">
+        <v>0</v>
+      </c>
+      <c r="M136" t="n">
+        <v>1</v>
+      </c>
+      <c r="N136" t="n">
+        <v>0</v>
+      </c>
+      <c r="O136" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q136" t="inlineStr">
+        <is>
+          <t>Conserva sólo las publicaciones sobre temas de interés público en el municipio de Morelia, Michoacán, México (seguridad, gobierno municipal o estatal, obras públicas, servicios como agua, basura, alumbrado, baches, movilidad y transporte, política y partidos, eventos y protestas, economía local, colonias y comunidades). Elimina: promoción de negocios, ventas y rentas, anuncios comerciales, saludos, publicaciones personales sin relevancia pública, y publicaciones que se refieran a otros lugares o cosas llamadas Morelia (calles llamadas Morelia en otras ciudades, el equipo de fútbol Atlético Morelia salvo que el tema sea de interés público local, Morelia como nombre de persona).</t>
+        </is>
+      </c>
+      <c r="S136" t="n">
+        <v>1</v>
+      </c>
+      <c r="T136" t="n">
+        <v>1</v>
+      </c>
+      <c r="U136" t="inlineStr">
+        <is>
+          <t>{"recent_posts": false, "enrich_author_after_likes": 100}</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>126</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>facebook_keyword_search</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>morelia_descifra</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Morelia keyword variants (round 1c, discovery)</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>morelia michoacán,ayuntamiento de morelia,gobierno de morelia,alfonso martínez morelia, morelia colonia,morelia baches,morelia agua,ooapas morelia,morelia obras, morelia seguridad,morelia policía,morelia transporte,morelia combis, morelia manifestación,morelia bloqueo,morelia bedolla,morelia morena,morelia pan, morelia tenencia,morelia alumbrado,morelia basura,morelia lluvias,morelia mercado, morelia vecinos,morelia centro histórico</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="K137" t="n">
+        <v>100</v>
+      </c>
+      <c r="L137" t="n">
+        <v>0</v>
+      </c>
+      <c r="M137" t="n">
+        <v>1</v>
+      </c>
+      <c r="N137" t="n">
+        <v>0</v>
+      </c>
+      <c r="O137" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q137" t="inlineStr">
+        <is>
+          <t>Conserva sólo las publicaciones sobre temas de interés público en el municipio de Morelia, Michoacán, México (seguridad, gobierno municipal o estatal, obras públicas, servicios como agua, basura, alumbrado, baches, movilidad y transporte, política y partidos, eventos y protestas, economía local, colonias y comunidades). Elimina: promoción de negocios, ventas y rentas, anuncios comerciales, saludos, publicaciones personales sin relevancia pública, y publicaciones que se refieran a otros lugares o cosas llamadas Morelia (calles llamadas Morelia en otras ciudades, el equipo de fútbol Atlético Morelia salvo que el tema sea de interés público local, Morelia como nombre de persona).</t>
+        </is>
+      </c>
+      <c r="S137" t="n">
+        <v>1</v>
+      </c>
+      <c r="T137" t="n">
+        <v>1</v>
+      </c>
+      <c r="U137" t="inlineStr">
+        <is>
+          <t>{"enrich_author_after_likes": 100}</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>127</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>morelia_descifra</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Gobierno de Morelia</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/MoreliaGob</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K138" t="n">
+        <v>100</v>
+      </c>
+      <c r="L138" t="n">
+        <v>1</v>
+      </c>
+      <c r="M138" t="n">
+        <v>1</v>
+      </c>
+      <c r="N138" t="n">
+        <v>0</v>
+      </c>
+      <c r="O138" t="n">
+        <v>15</v>
+      </c>
+      <c r="S138" t="n">
+        <v>0</v>
+      </c>
+      <c r="T138" t="n">
+        <v>1</v>
+      </c>
+      <c r="X138" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>128</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>morelia_descifra</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Alfonso Martínez Alcázar (alcalde)</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/AlfonsoMtz.Mx</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K139" t="n">
+        <v>50</v>
+      </c>
+      <c r="L139" t="n">
+        <v>1</v>
+      </c>
+      <c r="M139" t="n">
+        <v>1</v>
+      </c>
+      <c r="N139" t="n">
+        <v>0</v>
+      </c>
+      <c r="O139" t="n">
+        <v>15</v>
+      </c>
+      <c r="S139" t="n">
+        <v>0</v>
+      </c>
+      <c r="T139" t="n">
+        <v>1</v>
+      </c>
+      <c r="X139" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>129</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>morelia_descifra</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>OOAPAS Morelia</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/MoreliaOoapas</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K140" t="n">
+        <v>50</v>
+      </c>
+      <c r="L140" t="n">
+        <v>1</v>
+      </c>
+      <c r="M140" t="n">
+        <v>1</v>
+      </c>
+      <c r="N140" t="n">
+        <v>0</v>
+      </c>
+      <c r="O140" t="n">
+        <v>15</v>
+      </c>
+      <c r="S140" t="n">
+        <v>0</v>
+      </c>
+      <c r="T140" t="n">
+        <v>1</v>
+      </c>
+      <c r="X140" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>130</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>morelia_descifra</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Policía de Morelia</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/policiademorelia</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K141" t="n">
+        <v>50</v>
+      </c>
+      <c r="L141" t="n">
+        <v>1</v>
+      </c>
+      <c r="M141" t="n">
+        <v>1</v>
+      </c>
+      <c r="N141" t="n">
+        <v>0</v>
+      </c>
+      <c r="O141" t="n">
+        <v>15</v>
+      </c>
+      <c r="S141" t="n">
+        <v>0</v>
+      </c>
+      <c r="T141" t="n">
+        <v>1</v>
+      </c>
+      <c r="X141" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>131</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>morelia_descifra</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Secretaría del H. Ayuntamiento de Morelia</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/SecretariaAyuntamientoMorelia</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K142" t="n">
+        <v>30</v>
+      </c>
+      <c r="L142" t="n">
+        <v>1</v>
+      </c>
+      <c r="M142" t="n">
+        <v>1</v>
+      </c>
+      <c r="N142" t="n">
+        <v>0</v>
+      </c>
+      <c r="O142" t="n">
+        <v>15</v>
+      </c>
+      <c r="S142" t="n">
+        <v>0</v>
+      </c>
+      <c r="T142" t="n">
+        <v>1</v>
+      </c>
+      <c r="X142" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>132</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>morelia_descifra</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Secretaría de Desarrollo Urbano y Movilidad (Morelia)</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/DesarrolloUrbanoyMovilidad</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K143" t="n">
+        <v>30</v>
+      </c>
+      <c r="L143" t="n">
+        <v>1</v>
+      </c>
+      <c r="M143" t="n">
+        <v>1</v>
+      </c>
+      <c r="N143" t="n">
+        <v>0</v>
+      </c>
+      <c r="O143" t="n">
+        <v>15</v>
+      </c>
+      <c r="S143" t="n">
+        <v>0</v>
+      </c>
+      <c r="T143" t="n">
+        <v>1</v>
+      </c>
+      <c r="X143" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>133</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>morelia_descifra</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Gobierno de Michoacán</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/gobmichoacan</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K144" t="n">
+        <v>50</v>
+      </c>
+      <c r="L144" t="n">
+        <v>1</v>
+      </c>
+      <c r="M144" t="n">
+        <v>1</v>
+      </c>
+      <c r="N144" t="n">
+        <v>0</v>
+      </c>
+      <c r="O144" t="n">
+        <v>15</v>
+      </c>
+      <c r="S144" t="n">
+        <v>0</v>
+      </c>
+      <c r="T144" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>134</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>morelia_descifra</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>SCOP Michoacán (obras estatales)</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ScopMich</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K145" t="n">
+        <v>30</v>
+      </c>
+      <c r="L145" t="n">
+        <v>1</v>
+      </c>
+      <c r="M145" t="n">
+        <v>1</v>
+      </c>
+      <c r="N145" t="n">
+        <v>0</v>
+      </c>
+      <c r="O145" t="n">
+        <v>15</v>
+      </c>
+      <c r="S145" t="n">
+        <v>0</v>
+      </c>
+      <c r="T145" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>135</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>morelia_descifra</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Alarma Roja Morelia</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/AFMMORELIA</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K146" t="n">
+        <v>50</v>
+      </c>
+      <c r="L146" t="n">
+        <v>1</v>
+      </c>
+      <c r="M146" t="n">
+        <v>1</v>
+      </c>
+      <c r="N146" t="n">
+        <v>0</v>
+      </c>
+      <c r="O146" t="n">
+        <v>15</v>
+      </c>
+      <c r="S146" t="n">
+        <v>0</v>
+      </c>
+      <c r="T146" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>136</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>morelia_descifra</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>El Sol de Morelia</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ElSolDemorelia.OEM</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K147" t="n">
+        <v>50</v>
+      </c>
+      <c r="L147" t="n">
+        <v>1</v>
+      </c>
+      <c r="M147" t="n">
+        <v>1</v>
+      </c>
+      <c r="N147" t="n">
+        <v>0</v>
+      </c>
+      <c r="O147" t="n">
+        <v>15</v>
+      </c>
+      <c r="S147" t="n">
+        <v>0</v>
+      </c>
+      <c r="T147" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>137</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>morelia_descifra</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>LaPágina</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/LaPaginaNoticias</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K148" t="n">
+        <v>30</v>
+      </c>
+      <c r="L148" t="n">
+        <v>1</v>
+      </c>
+      <c r="M148" t="n">
+        <v>1</v>
+      </c>
+      <c r="N148" t="n">
+        <v>0</v>
+      </c>
+      <c r="O148" t="n">
+        <v>15</v>
+      </c>
+      <c r="S148" t="n">
+        <v>0</v>
+      </c>
+      <c r="T148" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>138</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>morelia_descifra</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Molinero Vial Morelia</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/people/Molinero-Vial-Morelia/100063642935437/</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K149" t="n">
+        <v>50</v>
+      </c>
+      <c r="L149" t="n">
+        <v>1</v>
+      </c>
+      <c r="M149" t="n">
+        <v>1</v>
+      </c>
+      <c r="N149" t="n">
+        <v>0</v>
+      </c>
+      <c r="O149" t="n">
+        <v>15</v>
+      </c>
+      <c r="S149" t="n">
+        <v>0</v>
+      </c>
+      <c r="T149" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>139</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>morelia_descifra</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>La Nota Roja</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/lanotarojamich</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K150" t="n">
+        <v>30</v>
+      </c>
+      <c r="L150" t="n">
+        <v>1</v>
+      </c>
+      <c r="M150" t="n">
+        <v>1</v>
+      </c>
+      <c r="N150" t="n">
+        <v>0</v>
+      </c>
+      <c r="O150" t="n">
+        <v>15</v>
+      </c>
+      <c r="S150" t="n">
+        <v>0</v>
+      </c>
+      <c r="T150" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>140</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>morelia_descifra</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Quadratín Michoacán</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/agenciaquadratin</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K151" t="n">
+        <v>50</v>
+      </c>
+      <c r="L151" t="n">
+        <v>1</v>
+      </c>
+      <c r="M151" t="n">
+        <v>1</v>
+      </c>
+      <c r="N151" t="n">
+        <v>0</v>
+      </c>
+      <c r="O151" t="n">
+        <v>15</v>
+      </c>
+      <c r="S151" t="n">
+        <v>0</v>
+      </c>
+      <c r="T151" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>141</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>morelia_descifra</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>MiMorelia.com</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/mimoreliacom</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K152" t="n">
+        <v>50</v>
+      </c>
+      <c r="L152" t="n">
+        <v>1</v>
+      </c>
+      <c r="M152" t="n">
+        <v>1</v>
+      </c>
+      <c r="N152" t="n">
+        <v>0</v>
+      </c>
+      <c r="O152" t="n">
+        <v>15</v>
+      </c>
+      <c r="S152" t="n">
+        <v>0</v>
+      </c>
+      <c r="T152" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>142</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>morelia_descifra</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Post Data</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/PostData.News</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K153" t="n">
+        <v>30</v>
+      </c>
+      <c r="L153" t="n">
+        <v>1</v>
+      </c>
+      <c r="M153" t="n">
+        <v>1</v>
+      </c>
+      <c r="N153" t="n">
+        <v>0</v>
+      </c>
+      <c r="O153" t="n">
+        <v>15</v>
+      </c>
+      <c r="S153" t="n">
+        <v>0</v>
+      </c>
+      <c r="T153" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>143</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>morelia_descifra</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>ACG</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/agenciacomunicaciongrafica</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K154" t="n">
+        <v>30</v>
+      </c>
+      <c r="L154" t="n">
+        <v>1</v>
+      </c>
+      <c r="M154" t="n">
+        <v>1</v>
+      </c>
+      <c r="N154" t="n">
+        <v>0</v>
+      </c>
+      <c r="O154" t="n">
+        <v>15</v>
+      </c>
+      <c r="S154" t="n">
+        <v>0</v>
+      </c>
+      <c r="T154" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>144</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>morelia_descifra</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Canal 13 Michoacán</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/Canal13Michoacan</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K155" t="n">
+        <v>30</v>
+      </c>
+      <c r="L155" t="n">
+        <v>1</v>
+      </c>
+      <c r="M155" t="n">
+        <v>1</v>
+      </c>
+      <c r="N155" t="n">
+        <v>0</v>
+      </c>
+      <c r="O155" t="n">
+        <v>15</v>
+      </c>
+      <c r="S155" t="n">
+        <v>0</v>
+      </c>
+      <c r="T155" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
tasks: Zitácuaro rows restored (146–158), Pinal/DL-15 rows 159–175, retired themes disabled; CURRENT_THEME env override; crawl-tasks DB design
- tasks.xlsx: the uncommitted Zitácuaro rows (124–136, 2026-08-17) were lost and
  their ids reused; re-appended from customer.yaml via customer_ops as 146–158.
  Pinal brief layer + DL-15 tracking rows 159–175; informe row 145 off; themes
  sjdr, orizaba, morelia_descifra, zona_fest, queretaro, mc, top_news,
  chepe_guerrero, felifer, efren_cuevas disabled (ledger:
  business_agent/docs/plans/task_cleanup_2026-10-05.json)
- run_searches.py: CURRENT_THEME=<theme> env var overrides the edited constant
- docs/db/crawl_tasks.md: userdb crawl_* tables design (org-scoped tasks, runs,
  per-call cost → usage_events, comments-on-demand); draft migration lives in
  media-backend-paid/docs/db/migrations/ (not applied)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tasks.xlsx
+++ b/tasks.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X155"/>
+  <dimension ref="A1:X186"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="19.6640625" customWidth="1" min="2" max="4"/>
@@ -1247,8 +1247,8 @@
       <c r="K11" t="n">
         <v>15</v>
       </c>
-      <c r="L11" t="b">
-        <v>1</v>
+      <c r="L11" t="n">
+        <v>0</v>
       </c>
       <c r="M11" t="b">
         <v>1</v>
@@ -1301,8 +1301,8 @@
       <c r="K12" t="n">
         <v>20</v>
       </c>
-      <c r="L12" t="b">
-        <v>1</v>
+      <c r="L12" t="n">
+        <v>0</v>
       </c>
       <c r="M12" t="b">
         <v>1</v>
@@ -1355,8 +1355,8 @@
       <c r="K13" t="n">
         <v>20</v>
       </c>
-      <c r="L13" t="b">
-        <v>1</v>
+      <c r="L13" t="n">
+        <v>0</v>
       </c>
       <c r="M13" t="b">
         <v>1</v>
@@ -1409,8 +1409,8 @@
       <c r="K14" t="n">
         <v>20</v>
       </c>
-      <c r="L14" t="b">
-        <v>1</v>
+      <c r="L14" t="n">
+        <v>0</v>
       </c>
       <c r="M14" t="b">
         <v>1</v>
@@ -1463,8 +1463,8 @@
       <c r="K15" t="n">
         <v>20</v>
       </c>
-      <c r="L15" t="b">
-        <v>1</v>
+      <c r="L15" t="n">
+        <v>0</v>
       </c>
       <c r="M15" t="b">
         <v>1</v>
@@ -1514,8 +1514,8 @@
       <c r="K16" t="n">
         <v>20</v>
       </c>
-      <c r="L16" t="b">
-        <v>1</v>
+      <c r="L16" t="n">
+        <v>0</v>
       </c>
       <c r="M16" t="b">
         <v>1</v>
@@ -1565,8 +1565,8 @@
       <c r="K17" t="n">
         <v>20</v>
       </c>
-      <c r="L17" t="b">
-        <v>1</v>
+      <c r="L17" t="n">
+        <v>0</v>
       </c>
       <c r="M17" t="b">
         <v>1</v>
@@ -1616,8 +1616,8 @@
       <c r="K18" t="n">
         <v>10</v>
       </c>
-      <c r="L18" t="b">
-        <v>1</v>
+      <c r="L18" t="n">
+        <v>0</v>
       </c>
       <c r="M18" t="b">
         <v>1</v>
@@ -1667,8 +1667,8 @@
       <c r="K19" t="n">
         <v>5</v>
       </c>
-      <c r="L19" t="b">
-        <v>1</v>
+      <c r="L19" t="n">
+        <v>0</v>
       </c>
       <c r="M19" t="b">
         <v>1</v>
@@ -1718,8 +1718,8 @@
       <c r="K20" t="n">
         <v>20</v>
       </c>
-      <c r="L20" t="b">
-        <v>1</v>
+      <c r="L20" t="n">
+        <v>0</v>
       </c>
       <c r="M20" t="b">
         <v>1</v>
@@ -1769,8 +1769,8 @@
       <c r="K21" t="n">
         <v>30</v>
       </c>
-      <c r="L21" t="b">
-        <v>1</v>
+      <c r="L21" t="n">
+        <v>0</v>
       </c>
       <c r="M21" t="b">
         <v>1</v>
@@ -1820,8 +1820,8 @@
       <c r="K22" t="n">
         <v>50</v>
       </c>
-      <c r="L22" t="b">
-        <v>1</v>
+      <c r="L22" t="n">
+        <v>0</v>
       </c>
       <c r="M22" t="b">
         <v>1</v>
@@ -1871,8 +1871,8 @@
       <c r="K23" t="n">
         <v>25</v>
       </c>
-      <c r="L23" t="b">
-        <v>1</v>
+      <c r="L23" t="n">
+        <v>0</v>
       </c>
       <c r="M23" t="b">
         <v>1</v>
@@ -1973,8 +1973,8 @@
       <c r="K25" t="n">
         <v>30</v>
       </c>
-      <c r="L25" t="b">
-        <v>1</v>
+      <c r="L25" t="n">
+        <v>0</v>
       </c>
       <c r="M25" t="b">
         <v>1</v>
@@ -6141,8 +6141,8 @@
       <c r="K86" t="n">
         <v>20</v>
       </c>
-      <c r="L86" t="b">
-        <v>1</v>
+      <c r="L86" t="n">
+        <v>0</v>
       </c>
       <c r="M86" t="b">
         <v>1</v>
@@ -6195,8 +6195,8 @@
       <c r="K87" t="n">
         <v>20</v>
       </c>
-      <c r="L87" t="b">
-        <v>1</v>
+      <c r="L87" t="n">
+        <v>0</v>
       </c>
       <c r="M87" t="b">
         <v>1</v>
@@ -6249,8 +6249,8 @@
       <c r="K88" t="n">
         <v>20</v>
       </c>
-      <c r="L88" t="b">
-        <v>1</v>
+      <c r="L88" t="n">
+        <v>0</v>
       </c>
       <c r="M88" t="b">
         <v>1</v>
@@ -6303,8 +6303,8 @@
       <c r="K89" t="n">
         <v>50</v>
       </c>
-      <c r="L89" t="b">
-        <v>1</v>
+      <c r="L89" t="n">
+        <v>0</v>
       </c>
       <c r="M89" t="b">
         <v>1</v>
@@ -6354,8 +6354,8 @@
       <c r="K90" t="n">
         <v>50</v>
       </c>
-      <c r="L90" t="b">
-        <v>1</v>
+      <c r="L90" t="n">
+        <v>0</v>
       </c>
       <c r="M90" t="b">
         <v>1</v>
@@ -6415,8 +6415,8 @@
       <c r="K91" t="n">
         <v>50</v>
       </c>
-      <c r="L91" t="b">
-        <v>1</v>
+      <c r="L91" t="n">
+        <v>0</v>
       </c>
       <c r="M91" t="b">
         <v>1</v>
@@ -6479,8 +6479,8 @@
       <c r="K92" t="n">
         <v>50</v>
       </c>
-      <c r="L92" t="b">
-        <v>1</v>
+      <c r="L92" t="n">
+        <v>0</v>
       </c>
       <c r="M92" t="b">
         <v>1</v>
@@ -6540,8 +6540,8 @@
       <c r="K93" t="n">
         <v>100</v>
       </c>
-      <c r="L93" t="b">
-        <v>1</v>
+      <c r="L93" t="n">
+        <v>0</v>
       </c>
       <c r="M93" t="b">
         <v>1</v>
@@ -6614,8 +6614,8 @@
       <c r="K94" t="n">
         <v>100</v>
       </c>
-      <c r="L94" t="b">
-        <v>1</v>
+      <c r="L94" t="n">
+        <v>0</v>
       </c>
       <c r="M94" t="b">
         <v>1</v>
@@ -6661,8 +6661,8 @@
       <c r="K95" t="n">
         <v>100</v>
       </c>
-      <c r="L95" t="b">
-        <v>1</v>
+      <c r="L95" t="n">
+        <v>0</v>
       </c>
       <c r="M95" t="b">
         <v>1</v>
@@ -6725,8 +6725,8 @@
       <c r="K96" t="n">
         <v>100</v>
       </c>
-      <c r="L96" t="b">
-        <v>1</v>
+      <c r="L96" t="n">
+        <v>0</v>
       </c>
       <c r="M96" t="b">
         <v>1</v>
@@ -6794,8 +6794,8 @@
       <c r="K97" t="n">
         <v>200</v>
       </c>
-      <c r="L97" t="b">
-        <v>1</v>
+      <c r="L97" t="n">
+        <v>0</v>
       </c>
       <c r="M97" t="b">
         <v>1</v>
@@ -6858,8 +6858,8 @@
       <c r="K98" t="n">
         <v>10</v>
       </c>
-      <c r="L98" t="b">
-        <v>1</v>
+      <c r="L98" t="n">
+        <v>0</v>
       </c>
       <c r="M98" t="b">
         <v>1</v>
@@ -6910,8 +6910,8 @@
       <c r="K99" t="n">
         <v>10</v>
       </c>
-      <c r="L99" t="b">
-        <v>1</v>
+      <c r="L99" t="n">
+        <v>0</v>
       </c>
       <c r="M99" t="b">
         <v>1</v>
@@ -6962,8 +6962,8 @@
       <c r="K100" t="n">
         <v>10</v>
       </c>
-      <c r="L100" t="b">
-        <v>1</v>
+      <c r="L100" t="n">
+        <v>0</v>
       </c>
       <c r="M100" t="b">
         <v>1</v>
@@ -7017,8 +7017,8 @@
       <c r="K101" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="L101" s="2" t="b">
-        <v>1</v>
+      <c r="L101" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="M101" s="2" t="b">
         <v>1</v>
@@ -7070,8 +7070,8 @@
       <c r="K102" t="n">
         <v>100</v>
       </c>
-      <c r="L102" t="b">
-        <v>1</v>
+      <c r="L102" t="n">
+        <v>0</v>
       </c>
       <c r="M102" t="b">
         <v>1</v>
@@ -7134,8 +7134,8 @@
       <c r="K103" t="n">
         <v>50</v>
       </c>
-      <c r="L103" t="b">
-        <v>1</v>
+      <c r="L103" t="n">
+        <v>0</v>
       </c>
       <c r="M103" t="b">
         <v>1</v>
@@ -7193,8 +7193,8 @@
       <c r="K104" t="n">
         <v>100</v>
       </c>
-      <c r="L104" t="b">
-        <v>1</v>
+      <c r="L104" t="n">
+        <v>0</v>
       </c>
       <c r="M104" t="b">
         <v>1</v>
@@ -7267,8 +7267,8 @@
       <c r="K105" t="n">
         <v>150</v>
       </c>
-      <c r="L105" t="b">
-        <v>1</v>
+      <c r="L105" t="n">
+        <v>0</v>
       </c>
       <c r="M105" t="b">
         <v>1</v>
@@ -7336,8 +7336,8 @@
       <c r="K106" t="n">
         <v>150</v>
       </c>
-      <c r="L106" t="b">
-        <v>1</v>
+      <c r="L106" t="n">
+        <v>0</v>
       </c>
       <c r="M106" t="b">
         <v>1</v>
@@ -7394,8 +7394,8 @@
       <c r="K107" t="n">
         <v>150</v>
       </c>
-      <c r="L107" t="b">
-        <v>1</v>
+      <c r="L107" t="n">
+        <v>0</v>
       </c>
       <c r="M107" t="b">
         <v>1</v>
@@ -7468,8 +7468,8 @@
       <c r="K108" t="n">
         <v>150</v>
       </c>
-      <c r="L108" t="b">
-        <v>1</v>
+      <c r="L108" t="n">
+        <v>0</v>
       </c>
       <c r="M108" t="b">
         <v>1</v>
@@ -7526,8 +7526,8 @@
       <c r="K109" t="n">
         <v>150</v>
       </c>
-      <c r="L109" t="b">
-        <v>1</v>
+      <c r="L109" t="n">
+        <v>0</v>
       </c>
       <c r="M109" t="b">
         <v>1</v>
@@ -7600,8 +7600,8 @@
       <c r="K110" t="n">
         <v>150</v>
       </c>
-      <c r="L110" t="b">
-        <v>1</v>
+      <c r="L110" t="n">
+        <v>0</v>
       </c>
       <c r="M110" t="b">
         <v>1</v>
@@ -7658,8 +7658,8 @@
       <c r="K111" t="n">
         <v>150</v>
       </c>
-      <c r="L111" t="b">
-        <v>1</v>
+      <c r="L111" t="n">
+        <v>0</v>
       </c>
       <c r="M111" t="b">
         <v>1</v>
@@ -7725,8 +7725,8 @@
       <c r="K112" t="n">
         <v>20</v>
       </c>
-      <c r="L112" t="b">
-        <v>1</v>
+      <c r="L112" t="n">
+        <v>0</v>
       </c>
       <c r="M112" t="b">
         <v>1</v>
@@ -7797,8 +7797,8 @@
       <c r="K113" t="n">
         <v>20</v>
       </c>
-      <c r="L113" t="b">
-        <v>1</v>
+      <c r="L113" t="n">
+        <v>0</v>
       </c>
       <c r="M113" t="b">
         <v>1</v>
@@ -7869,8 +7869,8 @@
       <c r="K114" t="n">
         <v>20</v>
       </c>
-      <c r="L114" t="b">
-        <v>1</v>
+      <c r="L114" t="n">
+        <v>0</v>
       </c>
       <c r="M114" t="b">
         <v>1</v>
@@ -7941,8 +7941,8 @@
       <c r="K115" t="n">
         <v>15</v>
       </c>
-      <c r="L115" t="b">
-        <v>1</v>
+      <c r="L115" t="n">
+        <v>0</v>
       </c>
       <c r="M115" t="b">
         <v>1</v>
@@ -8013,8 +8013,8 @@
       <c r="K116" t="n">
         <v>15</v>
       </c>
-      <c r="L116" t="b">
-        <v>1</v>
+      <c r="L116" t="n">
+        <v>0</v>
       </c>
       <c r="M116" t="b">
         <v>1</v>
@@ -8085,8 +8085,8 @@
       <c r="K117" t="n">
         <v>15</v>
       </c>
-      <c r="L117" t="b">
-        <v>1</v>
+      <c r="L117" t="n">
+        <v>0</v>
       </c>
       <c r="M117" t="b">
         <v>1</v>
@@ -8157,8 +8157,8 @@
       <c r="K118" t="n">
         <v>20</v>
       </c>
-      <c r="L118" t="b">
-        <v>1</v>
+      <c r="L118" t="n">
+        <v>0</v>
       </c>
       <c r="M118" t="b">
         <v>1</v>
@@ -8229,8 +8229,8 @@
       <c r="K119" t="n">
         <v>15</v>
       </c>
-      <c r="L119" t="b">
-        <v>1</v>
+      <c r="L119" t="n">
+        <v>0</v>
       </c>
       <c r="M119" t="b">
         <v>1</v>
@@ -8301,8 +8301,8 @@
       <c r="K120" t="n">
         <v>20</v>
       </c>
-      <c r="L120" t="b">
-        <v>1</v>
+      <c r="L120" t="n">
+        <v>0</v>
       </c>
       <c r="M120" t="b">
         <v>1</v>
@@ -8375,8 +8375,8 @@
       <c r="K121" t="n">
         <v>100</v>
       </c>
-      <c r="L121" t="b">
-        <v>1</v>
+      <c r="L121" t="n">
+        <v>0</v>
       </c>
       <c r="M121" t="b">
         <v>1</v>
@@ -8446,8 +8446,8 @@
       <c r="K122" t="n">
         <v>50</v>
       </c>
-      <c r="L122" t="b">
-        <v>1</v>
+      <c r="L122" t="n">
+        <v>0</v>
       </c>
       <c r="M122" t="b">
         <v>1</v>
@@ -8515,8 +8515,8 @@
       <c r="K123" t="n">
         <v>50</v>
       </c>
-      <c r="L123" t="b">
-        <v>1</v>
+      <c r="L123" t="n">
+        <v>0</v>
       </c>
       <c r="M123" t="b">
         <v>1</v>
@@ -8584,8 +8584,8 @@
       <c r="K124" t="n">
         <v>50</v>
       </c>
-      <c r="L124" t="b">
-        <v>1</v>
+      <c r="L124" t="n">
+        <v>0</v>
       </c>
       <c r="M124" t="b">
         <v>1</v>
@@ -8648,8 +8648,8 @@
       <c r="K125" t="n">
         <v>50</v>
       </c>
-      <c r="L125" t="b">
-        <v>1</v>
+      <c r="L125" t="n">
+        <v>0</v>
       </c>
       <c r="M125" t="b">
         <v>1</v>
@@ -8712,8 +8712,8 @@
       <c r="K126" t="n">
         <v>50</v>
       </c>
-      <c r="L126" t="b">
-        <v>1</v>
+      <c r="L126" t="n">
+        <v>0</v>
       </c>
       <c r="M126" t="b">
         <v>1</v>
@@ -8870,8 +8870,8 @@
       <c r="K129" t="n">
         <v>20</v>
       </c>
-      <c r="L129" t="b">
-        <v>1</v>
+      <c r="L129" t="n">
+        <v>0</v>
       </c>
       <c r="M129" t="b">
         <v>1</v>
@@ -9240,7 +9240,7 @@
         <v>50</v>
       </c>
       <c r="L135" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M135" t="n">
         <v>1</v>
@@ -9423,7 +9423,7 @@
         <v>100</v>
       </c>
       <c r="L138" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M138" t="n">
         <v>1</v>
@@ -9477,7 +9477,7 @@
         <v>50</v>
       </c>
       <c r="L139" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M139" t="n">
         <v>1</v>
@@ -9531,7 +9531,7 @@
         <v>50</v>
       </c>
       <c r="L140" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M140" t="n">
         <v>1</v>
@@ -9585,7 +9585,7 @@
         <v>50</v>
       </c>
       <c r="L141" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M141" t="n">
         <v>1</v>
@@ -9639,7 +9639,7 @@
         <v>30</v>
       </c>
       <c r="L142" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M142" t="n">
         <v>1</v>
@@ -9693,7 +9693,7 @@
         <v>30</v>
       </c>
       <c r="L143" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M143" t="n">
         <v>1</v>
@@ -9747,7 +9747,7 @@
         <v>50</v>
       </c>
       <c r="L144" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M144" t="n">
         <v>1</v>
@@ -9798,7 +9798,7 @@
         <v>30</v>
       </c>
       <c r="L145" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M145" t="n">
         <v>1</v>
@@ -9849,7 +9849,7 @@
         <v>50</v>
       </c>
       <c r="L146" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M146" t="n">
         <v>1</v>
@@ -9900,7 +9900,7 @@
         <v>50</v>
       </c>
       <c r="L147" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M147" t="n">
         <v>1</v>
@@ -9951,7 +9951,7 @@
         <v>30</v>
       </c>
       <c r="L148" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M148" t="n">
         <v>1</v>
@@ -10002,7 +10002,7 @@
         <v>50</v>
       </c>
       <c r="L149" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M149" t="n">
         <v>1</v>
@@ -10053,7 +10053,7 @@
         <v>30</v>
       </c>
       <c r="L150" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M150" t="n">
         <v>1</v>
@@ -10104,7 +10104,7 @@
         <v>50</v>
       </c>
       <c r="L151" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M151" t="n">
         <v>1</v>
@@ -10155,7 +10155,7 @@
         <v>50</v>
       </c>
       <c r="L152" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M152" t="n">
         <v>1</v>
@@ -10206,7 +10206,7 @@
         <v>30</v>
       </c>
       <c r="L153" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M153" t="n">
         <v>1</v>
@@ -10257,7 +10257,7 @@
         <v>30</v>
       </c>
       <c r="L154" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M154" t="n">
         <v>1</v>
@@ -10308,7 +10308,7 @@
         <v>30</v>
       </c>
       <c r="L155" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M155" t="n">
         <v>1</v>
@@ -10324,6 +10324,1748 @@
       </c>
       <c r="T155" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>145</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>facebook_keyword_search</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>pinal_amoles</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Informe de Gobierno Pinal de Amoles (keyword)</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>pinal de amoles informe de gobierno</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="K156" t="n">
+        <v>100</v>
+      </c>
+      <c r="L156" t="n">
+        <v>0</v>
+      </c>
+      <c r="M156" t="n">
+        <v>1</v>
+      </c>
+      <c r="N156" t="n">
+        <v>1</v>
+      </c>
+      <c r="O156" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q156" t="inlineStr">
+        <is>
+          <t>Conserva sólo las publicaciones sobre el Informe de Gobierno (V Informe) de la presidenta municipal de Pinal de Amoles, Querétaro, México, María Guadalupe «Lupita» Ramírez Plaza, o sobre las obras, programas y resultados que en él se informaron, y las reacciones a ese informe. Elimina informes de otros municipios o del gobierno del estado (por ejemplo el informe del gobernador Mauricio Kuri), promoción de negocios, ventas y publicaciones sin relación.</t>
+        </is>
+      </c>
+      <c r="S156" t="n">
+        <v>1</v>
+      </c>
+      <c r="T156" t="n">
+        <v>1</v>
+      </c>
+      <c r="U156" t="inlineStr">
+        <is>
+          <t>{"get_comments_after_likes": 10, "enrich_author_after_likes": 30}</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>146</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>facebook_keyword_search</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>zitacuaro</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Zitácuaro keyword</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>zitácuaro,zitacuaro</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K157" t="n">
+        <v>300</v>
+      </c>
+      <c r="L157" t="n">
+        <v>1</v>
+      </c>
+      <c r="M157" t="n">
+        <v>1</v>
+      </c>
+      <c r="N157" t="n">
+        <v>1</v>
+      </c>
+      <c r="O157" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q157" t="inlineStr">
+        <is>
+          <t>Conserva sólo las publicaciones sobre temas de interés público en el municipio de Zitácuaro, Michoacán, México (seguridad, gobierno, obras, servicios, política, eventos, economía local). Elimina promoción de negocios, ventas, anuncios comerciales, saludos y publicaciones personales sin relevancia pública.</t>
+        </is>
+      </c>
+      <c r="S157" t="n">
+        <v>1</v>
+      </c>
+      <c r="T157" t="n">
+        <v>1</v>
+      </c>
+      <c r="U157" t="inlineStr">
+        <is>
+          <t>{"get_comments_after_likes": 100, "enrich_author_after_likes": 100}</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>147</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>zitacuaro</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Ayuntamiento de Zitácuaro</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/ayuntamientozitacuaro</t>
+        </is>
+      </c>
+      <c r="F158" t="n">
+        <v>56421</v>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K158" t="n">
+        <v>50</v>
+      </c>
+      <c r="L158" t="n">
+        <v>1</v>
+      </c>
+      <c r="M158" t="n">
+        <v>1</v>
+      </c>
+      <c r="N158" t="n">
+        <v>1</v>
+      </c>
+      <c r="O158" t="n">
+        <v>15</v>
+      </c>
+      <c r="S158" t="n">
+        <v>0</v>
+      </c>
+      <c r="T158" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>148</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>zitacuaro</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Toño Ixtláhuac (alcalde)</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/JAntonioIxtlahuac</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K159" t="n">
+        <v>50</v>
+      </c>
+      <c r="L159" t="n">
+        <v>1</v>
+      </c>
+      <c r="M159" t="n">
+        <v>1</v>
+      </c>
+      <c r="N159" t="n">
+        <v>1</v>
+      </c>
+      <c r="O159" t="n">
+        <v>15</v>
+      </c>
+      <c r="S159" t="n">
+        <v>0</v>
+      </c>
+      <c r="T159" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>149</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>zitacuaro</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Es Zitácuaro</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/EsZitacuaro</t>
+        </is>
+      </c>
+      <c r="F160" t="n">
+        <v>245471</v>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K160" t="n">
+        <v>20</v>
+      </c>
+      <c r="L160" t="n">
+        <v>1</v>
+      </c>
+      <c r="M160" t="n">
+        <v>1</v>
+      </c>
+      <c r="N160" t="n">
+        <v>1</v>
+      </c>
+      <c r="O160" t="n">
+        <v>15</v>
+      </c>
+      <c r="S160" t="n">
+        <v>0</v>
+      </c>
+      <c r="T160" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>150</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>zitacuaro</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Digital Noticias Michoacán</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/DigitalNoticiasMich</t>
+        </is>
+      </c>
+      <c r="F161" t="n">
+        <v>143255</v>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K161" t="n">
+        <v>20</v>
+      </c>
+      <c r="L161" t="n">
+        <v>1</v>
+      </c>
+      <c r="M161" t="n">
+        <v>1</v>
+      </c>
+      <c r="N161" t="n">
+        <v>1</v>
+      </c>
+      <c r="O161" t="n">
+        <v>15</v>
+      </c>
+      <c r="S161" t="n">
+        <v>0</v>
+      </c>
+      <c r="T161" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>151</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>zitacuaro</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Marce Higareda de Paz</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/higaredadepaz</t>
+        </is>
+      </c>
+      <c r="F162" t="n">
+        <v>13099</v>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K162" t="n">
+        <v>15</v>
+      </c>
+      <c r="L162" t="n">
+        <v>1</v>
+      </c>
+      <c r="M162" t="n">
+        <v>1</v>
+      </c>
+      <c r="N162" t="n">
+        <v>1</v>
+      </c>
+      <c r="O162" t="n">
+        <v>15</v>
+      </c>
+      <c r="S162" t="n">
+        <v>0</v>
+      </c>
+      <c r="T162" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>152</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>zitacuaro</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Diálogo Directo (Gilberto Silva)</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/dialogo.directo.79</t>
+        </is>
+      </c>
+      <c r="F163" t="n">
+        <v>16876</v>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K163" t="n">
+        <v>15</v>
+      </c>
+      <c r="L163" t="n">
+        <v>1</v>
+      </c>
+      <c r="M163" t="n">
+        <v>1</v>
+      </c>
+      <c r="N163" t="n">
+        <v>1</v>
+      </c>
+      <c r="O163" t="n">
+        <v>15</v>
+      </c>
+      <c r="S163" t="n">
+        <v>0</v>
+      </c>
+      <c r="T163" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>153</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>zitacuaro</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Evolución En Línea Michoacán</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/EvolucionEnLineaMichoacan</t>
+        </is>
+      </c>
+      <c r="F164" t="n">
+        <v>3640</v>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K164" t="n">
+        <v>15</v>
+      </c>
+      <c r="L164" t="n">
+        <v>1</v>
+      </c>
+      <c r="M164" t="n">
+        <v>1</v>
+      </c>
+      <c r="N164" t="n">
+        <v>1</v>
+      </c>
+      <c r="O164" t="n">
+        <v>15</v>
+      </c>
+      <c r="S164" t="n">
+        <v>0</v>
+      </c>
+      <c r="T164" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>154</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>zitacuaro</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>El Clarín Diario de Zitácuaro</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/people/El-Clarin-Diario-de-Zit%C3%A1cuaro/100063494744425/</t>
+        </is>
+      </c>
+      <c r="F165" t="n">
+        <v>503</v>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K165" t="n">
+        <v>15</v>
+      </c>
+      <c r="L165" t="n">
+        <v>1</v>
+      </c>
+      <c r="M165" t="n">
+        <v>1</v>
+      </c>
+      <c r="N165" t="n">
+        <v>1</v>
+      </c>
+      <c r="O165" t="n">
+        <v>15</v>
+      </c>
+      <c r="S165" t="n">
+        <v>0</v>
+      </c>
+      <c r="T165" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>155</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>zitacuaro</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Periódico Milenio Zitácuaro</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/periodiconuevomileniomichoacan</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K166" t="n">
+        <v>30</v>
+      </c>
+      <c r="L166" t="n">
+        <v>1</v>
+      </c>
+      <c r="M166" t="n">
+        <v>1</v>
+      </c>
+      <c r="N166" t="n">
+        <v>1</v>
+      </c>
+      <c r="O166" t="n">
+        <v>15</v>
+      </c>
+      <c r="S166" t="n">
+        <v>0</v>
+      </c>
+      <c r="T166" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>156</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>zitacuaro</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Zitácuaro en la Red Noticias</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=100063548678123</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K167" t="n">
+        <v>30</v>
+      </c>
+      <c r="L167" t="n">
+        <v>1</v>
+      </c>
+      <c r="M167" t="n">
+        <v>1</v>
+      </c>
+      <c r="N167" t="n">
+        <v>1</v>
+      </c>
+      <c r="O167" t="n">
+        <v>15</v>
+      </c>
+      <c r="S167" t="n">
+        <v>0</v>
+      </c>
+      <c r="T167" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="n">
+        <v>157</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>zitacuaro</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>El Despertar</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/periodicoeldespertar</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K168" t="n">
+        <v>30</v>
+      </c>
+      <c r="L168" t="n">
+        <v>1</v>
+      </c>
+      <c r="M168" t="n">
+        <v>1</v>
+      </c>
+      <c r="N168" t="n">
+        <v>1</v>
+      </c>
+      <c r="O168" t="n">
+        <v>15</v>
+      </c>
+      <c r="S168" t="n">
+        <v>0</v>
+      </c>
+      <c r="T168" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>158</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>zitacuaro</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Buscabullas Zitacuaro</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/BuscabullasZ</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K169" t="n">
+        <v>30</v>
+      </c>
+      <c r="L169" t="n">
+        <v>1</v>
+      </c>
+      <c r="M169" t="n">
+        <v>1</v>
+      </c>
+      <c r="N169" t="n">
+        <v>1</v>
+      </c>
+      <c r="O169" t="n">
+        <v>15</v>
+      </c>
+      <c r="S169" t="n">
+        <v>0</v>
+      </c>
+      <c r="T169" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>159</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>facebook_keyword_search</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>pinal_amoles</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Pinal de Amoles keyword</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>pinal de amoles</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K170" t="n">
+        <v>100</v>
+      </c>
+      <c r="L170" t="n">
+        <v>1</v>
+      </c>
+      <c r="M170" t="n">
+        <v>1</v>
+      </c>
+      <c r="N170" t="n">
+        <v>1</v>
+      </c>
+      <c r="O170" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q170" t="inlineStr">
+        <is>
+          <t>Conserva sólo las publicaciones sobre temas de interés público en el municipio de Pinal de Amoles, en la Sierra Gorda de Querétaro, México, o en sus comunidades (seguridad, gobierno, obras, caminos, agua, servicios, programas, política, eventos, accidentes, clima, cultura). Elimina promoción de negocios, ventas, saludos, publicaciones personales sin relevancia pública y publicaciones sobre otros lugares con el mismo nombre.</t>
+        </is>
+      </c>
+      <c r="S170" t="n">
+        <v>1</v>
+      </c>
+      <c r="T170" t="n">
+        <v>1</v>
+      </c>
+      <c r="U170" t="inlineStr">
+        <is>
+          <t>{"get_comments_after_likes": 10, "enrich_author_after_likes": 30}</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>160</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>pinal_amoles</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Ayuntamiento de Pinal de Amoles (página oficial)</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/pinaldeamolesm</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K171" t="n">
+        <v>30</v>
+      </c>
+      <c r="L171" t="n">
+        <v>1</v>
+      </c>
+      <c r="M171" t="n">
+        <v>1</v>
+      </c>
+      <c r="N171" t="n">
+        <v>1</v>
+      </c>
+      <c r="O171" t="n">
+        <v>30</v>
+      </c>
+      <c r="S171" t="n">
+        <v>0</v>
+      </c>
+      <c r="T171" t="n">
+        <v>1</v>
+      </c>
+      <c r="U171" t="inlineStr">
+        <is>
+          <t>{"get_comments_after_likes": 10, "enrich_author_after_likes": 30}</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>161</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>pinal_amoles</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Lupita Ramírez Plaza (presidenta)</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/LupitaRPlaza</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K172" t="n">
+        <v>30</v>
+      </c>
+      <c r="L172" t="n">
+        <v>1</v>
+      </c>
+      <c r="M172" t="n">
+        <v>1</v>
+      </c>
+      <c r="N172" t="n">
+        <v>1</v>
+      </c>
+      <c r="O172" t="n">
+        <v>30</v>
+      </c>
+      <c r="S172" t="n">
+        <v>0</v>
+      </c>
+      <c r="T172" t="n">
+        <v>1</v>
+      </c>
+      <c r="U172" t="inlineStr">
+        <is>
+          <t>{"get_comments_after_likes": 10, "enrich_author_after_likes": 30}</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>162</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>pinal_amoles</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Iván Zárate (Inge Iván)</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/IvanZarateM</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="K173" t="n">
+        <v>40</v>
+      </c>
+      <c r="L173" t="n">
+        <v>1</v>
+      </c>
+      <c r="M173" t="n">
+        <v>1</v>
+      </c>
+      <c r="N173" t="n">
+        <v>1</v>
+      </c>
+      <c r="O173" t="n">
+        <v>30</v>
+      </c>
+      <c r="S173" t="n">
+        <v>0</v>
+      </c>
+      <c r="T173" t="n">
+        <v>1</v>
+      </c>
+      <c r="U173" t="inlineStr">
+        <is>
+          <t>{"get_comments_after_likes": 10, "enrich_author_after_likes": 30}</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>163</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>pinal_amoles</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Fernando Sánchez Gil (Arroyo Seco)</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/people/Fernando-S%C3%A1nchez/61558283724035/</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="K174" t="n">
+        <v>30</v>
+      </c>
+      <c r="L174" t="n">
+        <v>1</v>
+      </c>
+      <c r="M174" t="n">
+        <v>1</v>
+      </c>
+      <c r="N174" t="n">
+        <v>1</v>
+      </c>
+      <c r="O174" t="n">
+        <v>30</v>
+      </c>
+      <c r="S174" t="n">
+        <v>0</v>
+      </c>
+      <c r="T174" t="n">
+        <v>1</v>
+      </c>
+      <c r="U174" t="inlineStr">
+        <is>
+          <t>{"get_comments_after_likes": 10, "enrich_author_after_likes": 30}</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>164</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>pinal_amoles</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Astrid Ortega (Cadereyta)</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/AstridOrtegaV/</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="K175" t="n">
+        <v>30</v>
+      </c>
+      <c r="L175" t="n">
+        <v>1</v>
+      </c>
+      <c r="M175" t="n">
+        <v>1</v>
+      </c>
+      <c r="N175" t="n">
+        <v>1</v>
+      </c>
+      <c r="O175" t="n">
+        <v>30</v>
+      </c>
+      <c r="S175" t="n">
+        <v>0</v>
+      </c>
+      <c r="T175" t="n">
+        <v>1</v>
+      </c>
+      <c r="U175" t="inlineStr">
+        <is>
+          <t>{"get_comments_after_likes": 10, "enrich_author_after_likes": 30}</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>165</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>pinal_amoles</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Rubén Hernández (Jalpan)</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/p/Rub%C3%A9n-Hern%C3%A1ndez-61551688837412/</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="K176" t="n">
+        <v>30</v>
+      </c>
+      <c r="L176" t="n">
+        <v>1</v>
+      </c>
+      <c r="M176" t="n">
+        <v>1</v>
+      </c>
+      <c r="N176" t="n">
+        <v>1</v>
+      </c>
+      <c r="O176" t="n">
+        <v>30</v>
+      </c>
+      <c r="S176" t="n">
+        <v>0</v>
+      </c>
+      <c r="T176" t="n">
+        <v>1</v>
+      </c>
+      <c r="U176" t="inlineStr">
+        <is>
+          <t>{"get_comments_after_likes": 10, "enrich_author_after_likes": 30}</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>166</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>pinal_amoles</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Yuni Benítez (Landa)</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/p/Yuni-Ben%C3%ADtez-61557467575264/</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="K177" t="n">
+        <v>30</v>
+      </c>
+      <c r="L177" t="n">
+        <v>1</v>
+      </c>
+      <c r="M177" t="n">
+        <v>1</v>
+      </c>
+      <c r="N177" t="n">
+        <v>1</v>
+      </c>
+      <c r="O177" t="n">
+        <v>30</v>
+      </c>
+      <c r="S177" t="n">
+        <v>0</v>
+      </c>
+      <c r="T177" t="n">
+        <v>1</v>
+      </c>
+      <c r="U177" t="inlineStr">
+        <is>
+          <t>{"get_comments_after_likes": 10, "enrich_author_after_likes": 30}</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>167</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>pinal_amoles</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Carlos Manuel Ledesma (San Joaquín)</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/CarlosManuelLedesmaRobleSj/</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="K178" t="n">
+        <v>30</v>
+      </c>
+      <c r="L178" t="n">
+        <v>1</v>
+      </c>
+      <c r="M178" t="n">
+        <v>1</v>
+      </c>
+      <c r="N178" t="n">
+        <v>1</v>
+      </c>
+      <c r="O178" t="n">
+        <v>30</v>
+      </c>
+      <c r="S178" t="n">
+        <v>0</v>
+      </c>
+      <c r="T178" t="n">
+        <v>1</v>
+      </c>
+      <c r="U178" t="inlineStr">
+        <is>
+          <t>{"get_comments_after_likes": 10, "enrich_author_after_likes": 30}</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>168</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>pinal_amoles</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Blanca Benítez (diputada DL-15)</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/BlancaBenitezEstrada/</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="K179" t="n">
+        <v>30</v>
+      </c>
+      <c r="L179" t="n">
+        <v>1</v>
+      </c>
+      <c r="M179" t="n">
+        <v>1</v>
+      </c>
+      <c r="N179" t="n">
+        <v>1</v>
+      </c>
+      <c r="O179" t="n">
+        <v>30</v>
+      </c>
+      <c r="S179" t="n">
+        <v>0</v>
+      </c>
+      <c r="T179" t="n">
+        <v>1</v>
+      </c>
+      <c r="U179" t="inlineStr">
+        <is>
+          <t>{"get_comments_after_likes": 10, "enrich_author_after_likes": 30}</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>169</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>facebook_page_posts</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>pinal_amoles</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Agustín Dorantes (senador)</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/AgustinDoran/</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="K180" t="n">
+        <v>30</v>
+      </c>
+      <c r="L180" t="n">
+        <v>1</v>
+      </c>
+      <c r="M180" t="n">
+        <v>1</v>
+      </c>
+      <c r="N180" t="n">
+        <v>1</v>
+      </c>
+      <c r="O180" t="n">
+        <v>30</v>
+      </c>
+      <c r="S180" t="n">
+        <v>0</v>
+      </c>
+      <c r="T180" t="n">
+        <v>1</v>
+      </c>
+      <c r="U180" t="inlineStr">
+        <is>
+          <t>{"get_comments_after_likes": 10, "enrich_author_after_likes": 30}</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>170</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>facebook_keyword_search</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>pinal_amoles</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Jalpan de Serra keyword</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>jalpan de serra</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K181" t="n">
+        <v>100</v>
+      </c>
+      <c r="L181" t="n">
+        <v>1</v>
+      </c>
+      <c r="M181" t="n">
+        <v>1</v>
+      </c>
+      <c r="N181" t="n">
+        <v>1</v>
+      </c>
+      <c r="O181" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q181" t="inlineStr">
+        <is>
+          <t>Conserva sólo las publicaciones sobre temas de interés público en el municipio de Jalpan de Serra, en la Sierra Gorda de Querétaro, México, o en sus comunidades (seguridad, gobierno, obras, caminos, agua, servicios, programas, política, eventos, accidentes, clima, cultura). Elimina promoción de negocios, ventas, saludos, publicaciones personales sin relevancia pública y publicaciones sobre otros lugares con el mismo nombre.</t>
+        </is>
+      </c>
+      <c r="S181" t="n">
+        <v>1</v>
+      </c>
+      <c r="T181" t="n">
+        <v>1</v>
+      </c>
+      <c r="U181" t="inlineStr">
+        <is>
+          <t>{"get_comments_after_likes": 10, "enrich_author_after_likes": 30}</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>171</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>facebook_keyword_search</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>pinal_amoles</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Landa de Matamoros keyword</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>landa de matamoros</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K182" t="n">
+        <v>100</v>
+      </c>
+      <c r="L182" t="n">
+        <v>1</v>
+      </c>
+      <c r="M182" t="n">
+        <v>1</v>
+      </c>
+      <c r="N182" t="n">
+        <v>1</v>
+      </c>
+      <c r="O182" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q182" t="inlineStr">
+        <is>
+          <t>Conserva sólo las publicaciones sobre temas de interés público en el municipio de Landa de Matamoros, en la Sierra Gorda de Querétaro, México, o en sus comunidades (seguridad, gobierno, obras, caminos, agua, servicios, programas, política, eventos, accidentes, clima, cultura). Elimina promoción de negocios, ventas, saludos, publicaciones personales sin relevancia pública y publicaciones sobre otros lugares con el mismo nombre.</t>
+        </is>
+      </c>
+      <c r="S182" t="n">
+        <v>1</v>
+      </c>
+      <c r="T182" t="n">
+        <v>1</v>
+      </c>
+      <c r="U182" t="inlineStr">
+        <is>
+          <t>{"get_comments_after_likes": 10, "enrich_author_after_likes": 30}</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>172</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>facebook_keyword_search</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>pinal_amoles</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Cadereyta de Montes keyword</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>cadereyta de montes</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K183" t="n">
+        <v>100</v>
+      </c>
+      <c r="L183" t="n">
+        <v>1</v>
+      </c>
+      <c r="M183" t="n">
+        <v>1</v>
+      </c>
+      <c r="N183" t="n">
+        <v>1</v>
+      </c>
+      <c r="O183" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q183" t="inlineStr">
+        <is>
+          <t>Conserva sólo las publicaciones sobre temas de interés público en el municipio de Cadereyta de Montes, en la Sierra Gorda de Querétaro, México, o en sus comunidades (seguridad, gobierno, obras, caminos, agua, servicios, programas, política, eventos, accidentes, clima, cultura). Elimina promoción de negocios, ventas, saludos, publicaciones personales sin relevancia pública y publicaciones sobre otros lugares con el mismo nombre.</t>
+        </is>
+      </c>
+      <c r="S183" t="n">
+        <v>1</v>
+      </c>
+      <c r="T183" t="n">
+        <v>1</v>
+      </c>
+      <c r="U183" t="inlineStr">
+        <is>
+          <t>{"get_comments_after_likes": 10, "enrich_author_after_likes": 30}</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>173</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>facebook_keyword_search</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>pinal_amoles</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Arroyo Seco keyword</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>arroyo seco querétaro</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K184" t="n">
+        <v>100</v>
+      </c>
+      <c r="L184" t="n">
+        <v>1</v>
+      </c>
+      <c r="M184" t="n">
+        <v>1</v>
+      </c>
+      <c r="N184" t="n">
+        <v>1</v>
+      </c>
+      <c r="O184" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q184" t="inlineStr">
+        <is>
+          <t>Conserva sólo las publicaciones sobre temas de interés público en el municipio de Arroyo Seco, en la Sierra Gorda de Querétaro, México, o en sus comunidades (seguridad, gobierno, obras, caminos, agua, servicios, programas, política, eventos, accidentes, clima, cultura). Elimina promoción de negocios, ventas, saludos, publicaciones personales sin relevancia pública y publicaciones sobre otros lugares con el mismo nombre.</t>
+        </is>
+      </c>
+      <c r="S184" t="n">
+        <v>1</v>
+      </c>
+      <c r="T184" t="n">
+        <v>1</v>
+      </c>
+      <c r="U184" t="inlineStr">
+        <is>
+          <t>{"get_comments_after_likes": 10, "enrich_author_after_likes": 30}</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>174</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>facebook_keyword_search</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>pinal_amoles</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>San Joaquín keyword</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>san joaquín querétaro</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="K185" t="n">
+        <v>100</v>
+      </c>
+      <c r="L185" t="n">
+        <v>1</v>
+      </c>
+      <c r="M185" t="n">
+        <v>1</v>
+      </c>
+      <c r="N185" t="n">
+        <v>1</v>
+      </c>
+      <c r="O185" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q185" t="inlineStr">
+        <is>
+          <t>Conserva sólo las publicaciones sobre temas de interés público en el municipio de San Joaquín, en la Sierra Gorda de Querétaro, México, o en sus comunidades (seguridad, gobierno, obras, caminos, agua, servicios, programas, política, eventos, accidentes, clima, cultura). Elimina promoción de negocios, ventas, saludos, publicaciones personales sin relevancia pública y publicaciones sobre otros lugares con el mismo nombre.</t>
+        </is>
+      </c>
+      <c r="S185" t="n">
+        <v>1</v>
+      </c>
+      <c r="T185" t="n">
+        <v>1</v>
+      </c>
+      <c r="U185" t="inlineStr">
+        <is>
+          <t>{"get_comments_after_likes": 10, "enrich_author_after_likes": 30}</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>175</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>facebook_keyword_search</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>pinal_amoles</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Iván Zárate keyword</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>iván zárate</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="K186" t="n">
+        <v>60</v>
+      </c>
+      <c r="L186" t="n">
+        <v>1</v>
+      </c>
+      <c r="M186" t="n">
+        <v>1</v>
+      </c>
+      <c r="N186" t="n">
+        <v>1</v>
+      </c>
+      <c r="O186" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q186" t="inlineStr">
+        <is>
+          <t>Conserva sólo las publicaciones sobre Iván Zárate Muñoz («Inge Iván»), presidente del DIF municipal de Pinal de Amoles, Querétaro, esposo de la presidenta municipal Lupita Ramírez Plaza: sus actividades, declaraciones y las reacciones a ellas. Elimina publicaciones sobre otras personas llamadas Iván Zárate.</t>
+        </is>
+      </c>
+      <c r="S186" t="n">
+        <v>1</v>
+      </c>
+      <c r="T186" t="n">
+        <v>1</v>
+      </c>
+      <c r="U186" t="inlineStr">
+        <is>
+          <t>{"get_comments_after_likes": 10, "enrich_author_after_likes": 30}</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
tasks.xlsx: pinal_amoles + zitacuaro disabled — demo orgs now crawl from the local DB scheduler (rollout test, 2026-10-06)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tasks.xlsx
+++ b/tasks.xlsx
@@ -10291,7 +10291,7 @@
         <v>300</v>
       </c>
       <c r="L154" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M154" t="n">
         <v>1</v>
@@ -10355,7 +10355,7 @@
         <v>50</v>
       </c>
       <c r="L155" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M155" t="n">
         <v>1</v>
@@ -10406,7 +10406,7 @@
         <v>50</v>
       </c>
       <c r="L156" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M156" t="n">
         <v>1</v>
@@ -10460,7 +10460,7 @@
         <v>20</v>
       </c>
       <c r="L157" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M157" t="n">
         <v>1</v>
@@ -10514,7 +10514,7 @@
         <v>20</v>
       </c>
       <c r="L158" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M158" t="n">
         <v>1</v>
@@ -10568,7 +10568,7 @@
         <v>15</v>
       </c>
       <c r="L159" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M159" t="n">
         <v>1</v>
@@ -10622,7 +10622,7 @@
         <v>15</v>
       </c>
       <c r="L160" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M160" t="n">
         <v>1</v>
@@ -10676,7 +10676,7 @@
         <v>15</v>
       </c>
       <c r="L161" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M161" t="n">
         <v>1</v>
@@ -10730,7 +10730,7 @@
         <v>15</v>
       </c>
       <c r="L162" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M162" t="n">
         <v>1</v>
@@ -10781,7 +10781,7 @@
         <v>30</v>
       </c>
       <c r="L163" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M163" t="n">
         <v>1</v>
@@ -10832,7 +10832,7 @@
         <v>30</v>
       </c>
       <c r="L164" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M164" t="n">
         <v>1</v>
@@ -10883,7 +10883,7 @@
         <v>30</v>
       </c>
       <c r="L165" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M165" t="n">
         <v>1</v>
@@ -10934,7 +10934,7 @@
         <v>30</v>
       </c>
       <c r="L166" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M166" t="n">
         <v>1</v>
@@ -10985,7 +10985,7 @@
         <v>100</v>
       </c>
       <c r="L167" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M167" t="n">
         <v>1</v>
@@ -11046,7 +11046,7 @@
         <v>30</v>
       </c>
       <c r="L168" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M168" t="n">
         <v>1</v>
@@ -11102,7 +11102,7 @@
         <v>30</v>
       </c>
       <c r="L169" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M169" t="n">
         <v>1</v>
@@ -11158,7 +11158,7 @@
         <v>40</v>
       </c>
       <c r="L170" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M170" t="n">
         <v>1</v>
@@ -11214,7 +11214,7 @@
         <v>30</v>
       </c>
       <c r="L171" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M171" t="n">
         <v>1</v>
@@ -11270,7 +11270,7 @@
         <v>30</v>
       </c>
       <c r="L172" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M172" t="n">
         <v>1</v>
@@ -11326,7 +11326,7 @@
         <v>30</v>
       </c>
       <c r="L173" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M173" t="n">
         <v>1</v>
@@ -11382,7 +11382,7 @@
         <v>30</v>
       </c>
       <c r="L174" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M174" t="n">
         <v>1</v>
@@ -11438,7 +11438,7 @@
         <v>30</v>
       </c>
       <c r="L175" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M175" t="n">
         <v>1</v>
@@ -11494,7 +11494,7 @@
         <v>30</v>
       </c>
       <c r="L176" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M176" t="n">
         <v>1</v>
@@ -11550,7 +11550,7 @@
         <v>30</v>
       </c>
       <c r="L177" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M177" t="n">
         <v>1</v>
@@ -11606,7 +11606,7 @@
         <v>100</v>
       </c>
       <c r="L178" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M178" t="n">
         <v>1</v>
@@ -11667,7 +11667,7 @@
         <v>100</v>
       </c>
       <c r="L179" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M179" t="n">
         <v>1</v>
@@ -11728,7 +11728,7 @@
         <v>100</v>
       </c>
       <c r="L180" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M180" t="n">
         <v>1</v>
@@ -11789,7 +11789,7 @@
         <v>100</v>
       </c>
       <c r="L181" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M181" t="n">
         <v>1</v>
@@ -11850,7 +11850,7 @@
         <v>100</v>
       </c>
       <c r="L182" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M182" t="n">
         <v>1</v>
@@ -11911,7 +11911,7 @@
         <v>60</v>
       </c>
       <c r="L183" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M183" t="n">
         <v>1</v>

</xml_diff>